<commit_message>
Mother Encore Web Site Act 2 Pré-Release 13
</commit_message>
<xml_diff>
--- a/src/assets/xlsx/credits_roles.xlsx
+++ b/src/assets/xlsx/credits_roles.xlsx
@@ -14,13 +14,13 @@
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
     <author/>
-    <author>tc={0b55f6b3-32b9-440e-a546-4ad367432532}</author>
-    <author>tc={341c644b-ff95-41e3-8791-84c1988d5e3d}</author>
-    <author>tc={72ad567f-39dd-4177-8a28-a2bdb5aaa041}</author>
-    <author>tc={9c73f5f0-48c7-4040-ae78-1344b7c7a81a}</author>
-    <author>tc={a483b862-5bd5-42d1-adcf-521c739cd62d}</author>
-    <author>tc={c78b5377-bf6b-4f1d-84e4-fb3d77ce53c7}</author>
-    <author>tc={ef8286b8-02c6-4be0-b523-bd51dadceb09}</author>
+    <author>tc={04e5a08b-da2b-4e59-80c7-87afecc904ea}</author>
+    <author>tc={1a7c42b0-bd67-4179-8d70-af301b1d1bf0}</author>
+    <author>tc={1e079197-4907-4103-9445-8fa5ad0e60b3}</author>
+    <author>tc={60456f87-bbbf-4d96-a1bd-67215bd11204}</author>
+    <author>tc={77838b67-b96f-4acd-bfee-103eed8e3dae}</author>
+    <author>tc={bd383fd5-4995-4300-aeec-8db0b878c6cf}</author>
+    <author>tc={f233a673-fb30-4f5d-8bcc-5e533943f097}</author>
   </authors>
   <commentList>
     <comment authorId="0" ref="E5">
@@ -31,28 +31,37 @@
     <comment authorId="0" ref="B34">
       <text>
         <t xml:space="preserve">3 people
-he/him</t>
+she/her and he/him</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="E34">
+      <text>
+        <t xml:space="preserve">かんこくご　ほんやく</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="B63">
+      <text>
+        <t xml:space="preserve">he/him</t>
       </text>
     </comment>
     <comment authorId="0" ref="B30">
       <text>
-        <t xml:space="preserve">4 people
-he/him</t>
+        <t xml:space="preserve">Don't forget the final whitespace!</t>
       </text>
     </comment>
     <comment authorId="0" ref="E63">
       <text>
-        <t xml:space="preserve">プレイヤー</t>
+        <t xml:space="preserve">エグゼクティブ・プロデューサー</t>
       </text>
     </comment>
-    <comment authorId="0" ref="E30">
+    <comment authorId="0" ref="B59">
       <text>
-        <t xml:space="preserve">にほんご　ほんやく</t>
+        <t xml:space="preserve">Phil Sandhop, most likely he/him</t>
       </text>
     </comment>
     <comment authorId="0" ref="E59">
       <text>
-        <t xml:space="preserve">ほんやくしゃ</t>
+        <t xml:space="preserve">えいぶん　スクリプトライター</t>
       </text>
     </comment>
     <comment authorId="0" ref="E26">
@@ -60,9 +69,14 @@
         <t xml:space="preserve">プレイテスター</t>
       </text>
     </comment>
+    <comment authorId="0" ref="B55">
+      <text>
+        <t xml:space="preserve">Masao Tottori, supposedly he/him</t>
+      </text>
+    </comment>
     <comment authorId="0" ref="E55">
       <text>
-        <t xml:space="preserve">プログラマー</t>
+        <t xml:space="preserve">フィギュアモデリング</t>
       </text>
     </comment>
     <comment authorId="0" ref="E22">
@@ -72,7 +86,7 @@
     </comment>
     <comment authorId="0" ref="E51">
       <text>
-        <t xml:space="preserve">おんがく　プロデューサー</t>
+        <t xml:space="preserve">ゲームデザイナー</t>
       </text>
     </comment>
     <comment authorId="0" ref="E18">
@@ -85,9 +99,14 @@
         <t xml:space="preserve">アイテムアーティスト</t>
       </text>
     </comment>
+    <comment authorId="0" ref="B43">
+      <text>
+        <t xml:space="preserve">he/him</t>
+      </text>
+    </comment>
     <comment authorId="0" ref="E43">
       <text>
-        <t xml:space="preserve">スペシャルサンクス</t>
+        <t xml:space="preserve">たのしさのマネージャー</t>
       </text>
     </comment>
     <comment authorId="0" ref="E10">
@@ -97,8 +116,8 @@
     </comment>
     <comment authorId="0" ref="B39">
       <text>
-        <t xml:space="preserve">3 people
-she/her and he/him</t>
+        <t xml:space="preserve">2 people
+he/him and any pronouns</t>
       </text>
     </comment>
     <comment authorId="0" ref="E6">
@@ -117,24 +136,30 @@
         <t xml:space="preserve">MOTHER ENCOREスタッフロール</t>
       </text>
     </comment>
+    <comment authorId="0" ref="B31">
+      <text>
+        <t xml:space="preserve">4 people
+he/him</t>
+      </text>
+    </comment>
     <comment authorId="0" ref="E64">
       <text>
-        <t xml:space="preserve">プレイしていただき　ありがとうございました！</t>
+        <t xml:space="preserve">プレイヤー</t>
       </text>
     </comment>
     <comment authorId="0" ref="E31">
       <text>
-        <t xml:space="preserve">フランスご　ほんやく</t>
+        <t xml:space="preserve">にほんご　ほんやく</t>
       </text>
     </comment>
     <comment authorId="0" ref="E60">
       <text>
-        <t xml:space="preserve">スペシャルサンクス</t>
+        <t xml:space="preserve">ほんやくしゃ</t>
       </text>
     </comment>
     <comment authorId="0" ref="E56">
       <text>
-        <t xml:space="preserve">シナリオアシスタント</t>
+        <t xml:space="preserve">プログラマー</t>
       </text>
     </comment>
     <comment authorId="0" ref="E23">
@@ -144,17 +169,12 @@
     </comment>
     <comment authorId="0" ref="E52">
       <text>
-        <t xml:space="preserve">おんがく　こうか</t>
+        <t xml:space="preserve">おんがく　プロデューサー</t>
       </text>
     </comment>
     <comment authorId="0" ref="E19">
       <text>
         <t xml:space="preserve">プロモーションアーティスト</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="E48">
-      <text>
-        <t xml:space="preserve">げんさくスタッフ</t>
       </text>
     </comment>
     <comment authorId="0" ref="E15">
@@ -164,7 +184,7 @@
     </comment>
     <comment authorId="0" ref="E44">
       <text>
-        <t xml:space="preserve">ベリー・スペシャルサンクス</t>
+        <t xml:space="preserve">スペシャルサンクス</t>
       </text>
     </comment>
     <comment authorId="0" ref="E11">
@@ -174,7 +194,7 @@
     </comment>
     <comment authorId="0" ref="B40">
       <text>
-        <t xml:space="preserve">2 people
+        <t xml:space="preserve">3 people
 she/her and he/him</t>
       </text>
     </comment>
@@ -185,7 +205,7 @@
     </comment>
     <comment authorId="0" ref="B36">
       <text>
-        <t xml:space="preserve">2 people
+        <t xml:space="preserve">3 people
 he/him</t>
       </text>
     </comment>
@@ -194,30 +214,19 @@
         <t xml:space="preserve">プロジェクト・クリエイター</t>
       </text>
     </comment>
-    <comment authorId="0" ref="B32">
+    <comment authorId="0" ref="E65">
       <text>
-        <t xml:space="preserve">3 people
-he/him</t>
+        <t xml:space="preserve">プレイしていただき　ありがとうございました！</t>
       </text>
     </comment>
     <comment authorId="0" ref="E32">
       <text>
-        <t xml:space="preserve">イタリアご　ほんやく</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="B61">
-      <text>
-        <t xml:space="preserve">he/him</t>
+        <t xml:space="preserve">フランスご　ほんやく</t>
       </text>
     </comment>
     <comment authorId="0" ref="E61">
       <text>
-        <t xml:space="preserve">プロデューサー</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="E28">
-      <text>
-        <t xml:space="preserve">ほんやく</t>
+        <t xml:space="preserve">スペシャルサンクス</t>
       </text>
     </comment>
     <comment authorId="0" ref="B24">
@@ -227,7 +236,7 @@
     </comment>
     <comment authorId="0" ref="E57">
       <text>
-        <t xml:space="preserve">コーディネーター</t>
+        <t xml:space="preserve">シナリオアシスタント</t>
       </text>
     </comment>
     <comment authorId="0" ref="E24">
@@ -242,7 +251,7 @@
     </comment>
     <comment authorId="0" ref="E53">
       <text>
-        <t xml:space="preserve">キャラクターデザイナー</t>
+        <t xml:space="preserve">おんがく　こうか</t>
       </text>
     </comment>
     <comment authorId="0" ref="E20">
@@ -250,19 +259,19 @@
         <t xml:space="preserve">MOTHER ENCOREロゴデザイナー</t>
       </text>
     </comment>
-    <comment authorId="0" ref="B49">
-      <text>
-        <t xml:space="preserve">he/him</t>
-      </text>
-    </comment>
     <comment authorId="0" ref="E49">
       <text>
-        <t xml:space="preserve">ディレクター</t>
+        <t xml:space="preserve">げんさくスタッフ</t>
       </text>
     </comment>
     <comment authorId="0" ref="E16">
       <text>
         <t xml:space="preserve">バランスちょうせい</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="E45">
+      <text>
+        <t xml:space="preserve">ベリー・スペシャルサンクス</t>
       </text>
     </comment>
     <comment authorId="0" ref="E12">
@@ -272,8 +281,8 @@
     </comment>
     <comment authorId="0" ref="B41">
       <text>
-        <t xml:space="preserve">4 people
-he/him</t>
+        <t xml:space="preserve">2 people
+she/her and he/him</t>
       </text>
     </comment>
     <comment authorId="0" ref="E8">
@@ -283,18 +292,13 @@
     </comment>
     <comment authorId="0" ref="B37">
       <text>
-        <t xml:space="preserve">3 people
+        <t xml:space="preserve">2 people
 he/him</t>
       </text>
     </comment>
     <comment authorId="0" ref="B4">
       <text>
         <t xml:space="preserve">he/him</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="E37">
-      <text>
-        <t xml:space="preserve">ポーランドご　ほんやく</t>
       </text>
     </comment>
     <comment authorId="0" ref="E4">
@@ -305,12 +309,12 @@
     <comment authorId="0" ref="B33">
       <text>
         <t xml:space="preserve">3 people
-she/her and he/him</t>
+he/him</t>
       </text>
     </comment>
     <comment authorId="0" ref="E33">
       <text>
-        <t xml:space="preserve">かんこくご　ほんやく</t>
+        <t xml:space="preserve">イタリアご　ほんやく</t>
       </text>
     </comment>
     <comment authorId="0" ref="B62">
@@ -318,24 +322,19 @@
         <t xml:space="preserve">he/him</t>
       </text>
     </comment>
-    <comment authorId="0" ref="B29">
+    <comment authorId="0" ref="E62">
       <text>
-        <t xml:space="preserve">Don't forget the final whitespace!</t>
+        <t xml:space="preserve">プロデューサー</t>
       </text>
     </comment>
-    <comment authorId="0" ref="E62">
+    <comment authorId="0" ref="E29">
       <text>
-        <t xml:space="preserve">エグゼクティブ・プロデューサー</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="B58">
-      <text>
-        <t xml:space="preserve">Phil Sandhop, most likely he/him</t>
+        <t xml:space="preserve">ほんやく</t>
       </text>
     </comment>
     <comment authorId="0" ref="E58">
       <text>
-        <t xml:space="preserve">えいぶん　スクリプトライター</t>
+        <t xml:space="preserve">コーディネーター</t>
       </text>
     </comment>
     <comment authorId="0" ref="E25">
@@ -343,14 +342,9 @@
         <t xml:space="preserve">テスター</t>
       </text>
     </comment>
-    <comment authorId="0" ref="B54">
-      <text>
-        <t xml:space="preserve">Masao Tottori, supposedly he/him</t>
-      </text>
-    </comment>
     <comment authorId="0" ref="E54">
       <text>
-        <t xml:space="preserve">フィギュアモデリング</t>
+        <t xml:space="preserve">キャラクターデザイナー</t>
       </text>
     </comment>
     <comment authorId="0" ref="E21">
@@ -358,9 +352,14 @@
         <t xml:space="preserve">ライター</t>
       </text>
     </comment>
+    <comment authorId="0" ref="B50">
+      <text>
+        <t xml:space="preserve">he/him</t>
+      </text>
+    </comment>
     <comment authorId="0" ref="E50">
       <text>
-        <t xml:space="preserve">ゲームデザイナー</t>
+        <t xml:space="preserve">ディレクター</t>
       </text>
     </comment>
     <comment authorId="0" ref="E17">
@@ -375,12 +374,8 @@
     </comment>
     <comment authorId="0" ref="B42">
       <text>
-        <t xml:space="preserve">he/him</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="E42">
-      <text>
-        <t xml:space="preserve">たのしさのマネージャー</t>
+        <t xml:space="preserve">4 people
+he/him</t>
       </text>
     </comment>
     <comment authorId="0" ref="E9">
@@ -390,11 +385,28 @@
     </comment>
     <comment authorId="0" ref="B38">
       <text>
-        <t xml:space="preserve">2 people
-he/him and any pronouns</t>
+        <t xml:space="preserve">3 people
+he/him</t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{0b55f6b3-32b9-440e-a546-4ad367432532}" ref="K36">
+    <comment authorId="0" ref="E38">
+      <text>
+        <t xml:space="preserve">ポーランドご　ほんやく</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{04e5a08b-da2b-4e59-80c7-87afecc904ea}" ref="K36">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Needs update for 2 people
+</t>
+      </text>
+    </comment>
+    <comment authorId="2" xr:uid="{1a7c42b0-bd67-4179-8d70-af301b1d1bf0}" ref="K37">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -406,7 +418,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{341c644b-ff95-41e3-8791-84c1988d5e3d}" ref="K34">
+    <comment authorId="3" xr:uid="{1e079197-4907-4103-9445-8fa5ad0e60b3}" ref="K35">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -418,7 +430,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="3" xr:uid="{72ad567f-39dd-4177-8a28-a2bdb5aaa041}" ref="B3">
+    <comment authorId="4" xr:uid="{60456f87-bbbf-4d96-a1bd-67215bd11204}" ref="B3">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -427,7 +439,19 @@
 </t>
       </text>
     </comment>
-    <comment authorId="4" xr:uid="{9c73f5f0-48c7-4040-ae78-1344b7c7a81a}" ref="K33">
+    <comment authorId="5" xr:uid="{77838b67-b96f-4acd-bfee-103eed8e3dae}" ref="J35">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Too long line, cuts right after "Łacińsk"
+</t>
+      </text>
+    </comment>
+    <comment authorId="6" xr:uid="{bd383fd5-4995-4300-aeec-8db0b878c6cf}" ref="K34">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -440,31 +464,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="5" xr:uid="{a483b862-5bd5-42d1-adcf-521c739cd62d}" ref="K35">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Needs update for 2 people
-</t>
-      </text>
-    </comment>
-    <comment authorId="6" xr:uid="{c78b5377-bf6b-4f1d-84e4-fb3d77ce53c7}" ref="J34">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Too long line, cuts right after "Łacińsk"
-</t>
-      </text>
-    </comment>
-    <comment authorId="7" xr:uid="{ef8286b8-02c6-4be0-b523-bd51dadceb09}" ref="B66">
+    <comment authorId="7" xr:uid="{f233a673-fb30-4f5d-8bcc-5e533943f097}" ref="B67">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -478,7 +478,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="756">
   <si>
     <t>key</t>
   </si>
@@ -1317,6 +1317,30 @@
     <t>游戏测试员</t>
   </si>
   <si>
+    <t>CREDITS_WEBSITE_PROGRAMMER</t>
+  </si>
+  <si>
+    <t>WEBSITE PROGRAMMERS</t>
+  </si>
+  <si>
+    <t>DÉVELLOPEURS DU SITE WEB</t>
+  </si>
+  <si>
+    <t>PROGRAMADORES DE SITIO WEB</t>
+  </si>
+  <si>
+    <t>PROGRAMIŚCI STRONY INTERNETOWEJ</t>
+  </si>
+  <si>
+    <t>WEBSEITEN-PROGRAMMIERER</t>
+  </si>
+  <si>
+    <t>ВЕБ-ПРОГРАММИСТЫ</t>
+  </si>
+  <si>
+    <t>网站程序</t>
+  </si>
+  <si>
     <t>CREDITS_TRANSLATION_MANAGER</t>
   </si>
   <si>
@@ -1338,7 +1362,7 @@
     <t>MANAGER DS. TŁUMACZEŃ</t>
   </si>
   <si>
-    <t>ÜBERSETZUNGSMANAGER</t>
+    <t>ÜBERSETZUNGSMANAGERIN</t>
   </si>
   <si>
     <t>МЕНЕДЖЕРЫ ПО ПЕРЕВОДАМ</t>
@@ -2606,7 +2630,7 @@
     <t>MOTHER ENCORE ACTE 1</t>
   </si>
   <si>
-    <t>TITOLI DI CODA ATTO 1</t>
+    <t>MOTHER ENCORE ATTO 1</t>
   </si>
   <si>
     <t>MOTHER ENCORE ACT1</t>
@@ -2639,7 +2663,7 @@
     <t>MOTHER ENCORE ACTE 2</t>
   </si>
   <si>
-    <t>TITOLI DI CODA ATTO 2</t>
+    <t>MOTHER ENCORE ATTO 2</t>
   </si>
   <si>
     <t>MOTHER ENCORE ACT2</t>
@@ -2681,7 +2705,7 @@
     <t>CRÉDITOS DA EQUIPE</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t>NAPISY KOŃCOWE</t>
   </si>
   <si>
     <t xml:space="preserve"> MITWIRKENDE</t>
@@ -2980,7 +3004,7 @@
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -2989,10 +3013,10 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -3004,7 +3028,7 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -3094,18 +3118,18 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Andy" id="{61e68ad2-f470-4937-8df8-fbb3e3da150b}" providerId="google-sheets"/>
-  <x18tc:person displayName="tc={08c2a535-b40d-4407-a54b-cb888ceebf26}" id="{54805936-8925-4f0b-a090-872408d94ef8}" providerId="google-sheets"/>
-  <x18tc:person displayName="tc={177d0a9e-f1f1-4ce6-be59-2b06cc365826}" id="{b61ee0e0-7b56-4c33-935e-f1420da8a52f}" providerId="google-sheets"/>
-  <x18tc:person displayName="tc={6737e3ce-96c6-488e-b0fb-70ed28d3c853}" id="{206c5ab3-90ef-4032-93ee-be43f32594fe}" providerId="google-sheets"/>
-  <x18tc:person displayName="tc={04c50c11-f702-436b-83cc-b7cc9fcef5c8}" id="{a383d35c-8d5d-4e2a-b671-e09e1605477a}" providerId="google-sheets"/>
-  <x18tc:person displayName="tc={a4284126-3e21-4fd6-b5bd-b042e323a701}" id="{75912930-2680-49f7-8676-eb89a23cecbc}" providerId="google-sheets"/>
-  <x18tc:person displayName="Danionel" id="{4e667a47-6342-400d-a397-64c7b20beef5}" providerId="google-sheets"/>
+  <x18tc:person displayName="Andy" id="{10ab281f-a151-41dc-8aaf-becb25b01a90}" providerId="google-sheets"/>
+  <x18tc:person displayName="tc={08c2a535-b40d-4407-a54b-cb888ceebf26}" id="{25a095f6-c4d1-4be2-ad36-a2f49cc34171}" providerId="google-sheets"/>
+  <x18tc:person displayName="tc={177d0a9e-f1f1-4ce6-be59-2b06cc365826}" id="{2641dc07-92da-44fe-80f0-28a2b0aee133}" providerId="google-sheets"/>
+  <x18tc:person displayName="tc={6737e3ce-96c6-488e-b0fb-70ed28d3c853}" id="{fe177049-05ac-4e23-96cf-3e43e63a1ae7}" providerId="google-sheets"/>
+  <x18tc:person displayName="tc={04c50c11-f702-436b-83cc-b7cc9fcef5c8}" id="{58cd9450-3c64-4eec-a904-c491f0e0b225}" providerId="google-sheets"/>
+  <x18tc:person displayName="tc={a4284126-3e21-4fd6-b5bd-b042e323a701}" id="{402daf81-0dc5-4899-ad3e-3b7fed17def7}" providerId="google-sheets"/>
+  <x18tc:person displayName="Danionel" id="{d24cb8d1-5f88-4660-bc5a-20409d23f659}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:N75" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:N76" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="14">
     <tableColumn name="key" id="1"/>
     <tableColumn name="en" id="2"/>
@@ -3322,10 +3346,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B66" dT="2026-05-27T04:15:36.00" personId="{61e68ad2-f470-4937-8df8-fbb3e3da150b}" id="{ef8286b8-02c6-4be0-b523-bd51dadceb09}" done="0">
+  <x18tc:threadedComment ref="B67" dT="2026-05-27T04:15:36.00" personId="{10ab281f-a151-41dc-8aaf-becb25b01a90}" id="{f233a673-fb30-4f5d-8bcc-5e533943f097}" done="0">
     <x18tc:text xml:space="preserve">Added "ACT 2"</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="K36" dT="2026-02-10T15:18:23.00" personId="{206c5ab3-90ef-4032-93ee-be43f32594fe}" id="{0b55f6b3-32b9-440e-a546-4ad367432532}" done="0">
+  <x18tc:threadedComment ref="K37" dT="2026-02-10T15:18:23.00" personId="{fe177049-05ac-4e23-96cf-3e43e63a1ae7}" id="{1a7c42b0-bd67-4179-8d70-af301b1d1bf0}" done="0">
     <x18tc:text xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
@@ -3337,7 +3361,7 @@
       </ext>
     </x18tc:extLst>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="K34" dT="2026-02-10T15:18:23.00" personId="{a383d35c-8d5d-4e2a-b671-e09e1605477a}" id="{341c644b-ff95-41e3-8791-84c1988d5e3d}" done="0">
+  <x18tc:threadedComment ref="K35" dT="2026-02-10T15:18:23.00" personId="{58cd9450-3c64-4eec-a904-c491f0e0b225}" id="{1e079197-4907-4103-9445-8fa5ad0e60b3}" done="0">
     <x18tc:text xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
@@ -3349,7 +3373,7 @@
       </ext>
     </x18tc:extLst>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="K33" dT="2026-02-10T15:18:23.00" personId="{75912930-2680-49f7-8676-eb89a23cecbc}" id="{9c73f5f0-48c7-4040-ae78-1344b7c7a81a}" done="0">
+  <x18tc:threadedComment ref="K34" dT="2026-02-10T15:18:23.00" personId="{402daf81-0dc5-4899-ad3e-3b7fed17def7}" id="{bd383fd5-4995-4300-aeec-8db0b878c6cf}" done="0">
     <x18tc:text xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
@@ -3362,7 +3386,7 @@
       </ext>
     </x18tc:extLst>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="K35" dT="2026-02-10T15:18:23.00" personId="{b61ee0e0-7b56-4c33-935e-f1420da8a52f}" id="{a483b862-5bd5-42d1-adcf-521c739cd62d}" done="0">
+  <x18tc:threadedComment ref="K36" dT="2026-02-10T15:18:23.00" personId="{2641dc07-92da-44fe-80f0-28a2b0aee133}" id="{04e5a08b-da2b-4e59-80c7-87afecc904ea}" done="0">
     <x18tc:text xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
@@ -3374,10 +3398,10 @@
       </ext>
     </x18tc:extLst>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="B3" dT="2026-03-06T16:37:41.00" personId="{4e667a47-6342-400d-a397-64c7b20beef5}" id="{72ad567f-39dd-4177-8a28-a2bdb5aaa041}" done="0">
+  <x18tc:threadedComment ref="B3" dT="2026-03-06T16:37:41.00" personId="{d24cb8d1-5f88-4660-bc5a-20409d23f659}" id="{60456f87-bbbf-4d96-a1bd-67215bd11204}" done="0">
     <x18tc:text xml:space="preserve">Sam uses she/her pronouns now, change your translations if needed</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="J34" dT="2026-02-10T15:18:23.00" personId="{54805936-8925-4f0b-a090-872408d94ef8}" id="{c78b5377-bf6b-4f1d-84e4-fb3d77ce53c7}" done="1">
+  <x18tc:threadedComment ref="J35" dT="2026-02-10T15:18:23.00" personId="{25a095f6-c4d1-4be2-ad36-a2f49cc34171}" id="{77838b67-b96f-4acd-bfee-103eed8e3dae}" done="1">
     <x18tc:text xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
@@ -4917,47 +4941,37 @@
       <c r="AB26" s="4"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="G27" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="G27" s="2" t="s">
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="H27" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="I27" s="2" t="s">
+      <c r="K27" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="J27" s="2" t="s">
+      <c r="L27" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="K27" s="2" t="s">
+      <c r="M27" s="3"/>
+      <c r="N27" s="5" t="s">
         <v>286</v>
-      </c>
-      <c r="L27" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="N27" s="5" t="s">
-        <v>289</v>
       </c>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
@@ -4976,46 +4990,46 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="E28" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="H28" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="I28" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="J28" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="G28" s="2" t="s">
+      <c r="K28" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="H28" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="I28" s="2" t="s">
+      <c r="L28" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="J28" s="2" t="s">
+      <c r="M28" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="K28" s="2" t="s">
+      <c r="N28" s="5" t="s">
         <v>297</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="N28" s="5" t="s">
-        <v>300</v>
       </c>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
@@ -5034,42 +5048,42 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="B29" s="12" t="s">
+      <c r="E29" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="H29" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="I29" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="D29" s="12" t="s">
-        <v>302</v>
-      </c>
-      <c r="E29" s="12" t="s">
-        <v>302</v>
-      </c>
-      <c r="F29" s="12" t="s">
-        <v>302</v>
-      </c>
-      <c r="G29" s="12" t="s">
+      <c r="J29" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="H29" s="12" t="s">
-        <v>304</v>
-      </c>
-      <c r="I29" s="12" t="s">
+      <c r="K29" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="J29" s="12" t="s">
+      <c r="L29" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="K29" s="12" t="s">
-        <v>302</v>
-      </c>
-      <c r="L29" s="12" t="s">
-        <v>307</v>
-      </c>
-      <c r="M29" s="12" t="s">
+      <c r="M29" s="2" t="s">
         <v>307</v>
       </c>
       <c r="N29" s="5" t="s">
@@ -5094,44 +5108,44 @@
       <c r="A30" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="12" t="s">
         <v>310</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="G30" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="H30" s="12" t="s">
+        <v>312</v>
+      </c>
+      <c r="I30" s="12" t="s">
         <v>313</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="J30" s="12" t="s">
         <v>314</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="K30" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="L30" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="M30" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="N30" s="5" t="s">
         <v>316</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="M30" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="N30" s="5" t="s">
-        <v>322</v>
       </c>
       <c r="O30" s="4"/>
       <c r="P30" s="4"/>
@@ -5150,46 +5164,46 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="H31" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="I31" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="J31" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="K31" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="L31" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="M31" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="N31" s="5" t="s">
         <v>330</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="N31" s="5" t="s">
-        <v>336</v>
       </c>
       <c r="O31" s="4"/>
       <c r="P31" s="4"/>
@@ -5208,46 +5222,46 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="G32" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="H32" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="I32" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="J32" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="K32" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="L32" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="M32" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="H32" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="I32" s="3" t="s">
+      <c r="N32" s="5" t="s">
         <v>344</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="N32" s="5" t="s">
-        <v>349</v>
       </c>
       <c r="O32" s="4"/>
       <c r="P32" s="4"/>
@@ -5266,46 +5280,46 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="H33" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="I33" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="J33" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="K33" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="L33" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="M33" s="2" t="s">
         <v>356</v>
       </c>
-      <c r="H33" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="I33" s="3" t="s">
+      <c r="N33" s="5" t="s">
         <v>357</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>359</v>
-      </c>
-      <c r="L33" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>361</v>
-      </c>
-      <c r="N33" s="5" t="s">
-        <v>362</v>
       </c>
       <c r="O33" s="4"/>
       <c r="P33" s="4"/>
@@ -5324,46 +5338,46 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>361</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="H34" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="I34" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="J34" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="K34" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="G34" s="2" t="s">
+      <c r="L34" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="H34" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="I34" s="3" t="s">
+      <c r="M34" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="J34" s="2" t="s">
+      <c r="N34" s="5" t="s">
         <v>370</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>373</v>
-      </c>
-      <c r="N34" s="5" t="s">
-        <v>374</v>
       </c>
       <c r="O34" s="4"/>
       <c r="P34" s="4"/>
@@ -5382,46 +5396,46 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="F35" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="H35" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="I35" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="J35" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="K35" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="F35" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="G35" s="2" t="s">
+      <c r="L35" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="H35" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="I35" s="3" t="s">
+      <c r="M35" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="J35" s="2" t="s">
+      <c r="N35" s="5" t="s">
         <v>382</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="M35" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="N35" s="5" t="s">
-        <v>386</v>
       </c>
       <c r="O35" s="4"/>
       <c r="P35" s="4"/>
@@ -5440,46 +5454,46 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>386</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="F36" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="H36" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="I36" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="J36" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="K36" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="F36" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="G36" s="2" t="s">
+      <c r="L36" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="H36" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="I36" s="3" t="s">
+      <c r="M36" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="J36" s="2" t="s">
+      <c r="N36" s="5" t="s">
         <v>394</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="N36" s="5" t="s">
-        <v>398</v>
       </c>
       <c r="O36" s="4"/>
       <c r="P36" s="4"/>
@@ -5498,46 +5512,46 @@
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>398</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="F37" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="G37" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="H37" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="I37" s="3" t="s">
         <v>401</v>
       </c>
-      <c r="D37" s="13" t="s">
+      <c r="J37" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="G37" s="2" t="s">
+      <c r="K37" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="H37" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="I37" s="3" t="s">
+      <c r="L37" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="J37" s="2" t="s">
+      <c r="M37" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="N37" s="5" t="s">
         <v>406</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="N37" s="5" t="s">
-        <v>409</v>
       </c>
       <c r="O37" s="4"/>
       <c r="P37" s="4"/>
@@ -5556,46 +5570,46 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="D38" s="13" t="s">
         <v>410</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="E38" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="H38" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="I38" s="3" t="s">
         <v>412</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="J38" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="E38" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="G38" s="2" t="s">
+      <c r="K38" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="H38" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="I38" s="3" t="s">
+      <c r="L38" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="J38" s="2" t="s">
+      <c r="M38" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="K38" s="2" t="s">
+      <c r="N38" s="5" t="s">
         <v>417</v>
-      </c>
-      <c r="L38" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="N38" s="5" t="s">
-        <v>420</v>
       </c>
       <c r="O38" s="4"/>
       <c r="P38" s="4"/>
@@ -5614,46 +5628,46 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="D39" s="13" t="s">
         <v>421</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="E39" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="G39" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="H39" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="I39" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="J39" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="E39" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="G39" s="2" t="s">
+      <c r="K39" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="H39" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="I39" s="3" t="s">
+      <c r="L39" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="J39" s="2" t="s">
+      <c r="M39" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="K39" s="2" t="s">
+      <c r="N39" s="5" t="s">
         <v>428</v>
-      </c>
-      <c r="L39" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="M39" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="N39" s="5" t="s">
-        <v>431</v>
       </c>
       <c r="O39" s="4"/>
       <c r="P39" s="4"/>
@@ -5672,46 +5686,46 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="E40" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="H40" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="I40" s="3" t="s">
         <v>434</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="J40" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="G40" s="2" t="s">
+      <c r="K40" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="H40" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="I40" s="3" t="s">
+      <c r="L40" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="J40" s="2" t="s">
+      <c r="M40" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="K40" s="2" t="s">
+      <c r="N40" s="5" t="s">
         <v>439</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="N40" s="5" t="s">
-        <v>442</v>
       </c>
       <c r="O40" s="4"/>
       <c r="P40" s="4"/>
@@ -5729,47 +5743,47 @@
       <c r="AB40" s="4"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="14" t="s">
+      <c r="A41" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="B41" s="15" t="s">
+      <c r="E41" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="H41" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="I41" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="J41" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>444</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>444</v>
-      </c>
-      <c r="G41" s="3" t="s">
+      <c r="K41" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="H41" s="3" t="s">
-        <v>447</v>
-      </c>
-      <c r="I41" s="3" t="s">
+      <c r="L41" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="J41" s="3" t="s">
+      <c r="M41" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="K41" s="3" t="s">
+      <c r="N41" s="5" t="s">
         <v>450</v>
-      </c>
-      <c r="L41" s="3" t="s">
-        <v>451</v>
-      </c>
-      <c r="M41" s="3" t="s">
-        <v>452</v>
-      </c>
-      <c r="N41" s="5" t="s">
-        <v>453</v>
       </c>
       <c r="O41" s="4"/>
       <c r="P41" s="4"/>
@@ -5787,47 +5801,47 @@
       <c r="AB41" s="4"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>452</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="D42" s="3" t="s">
         <v>454</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="E42" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="G42" s="3" t="s">
         <v>455</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="H42" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="I42" s="3" t="s">
         <v>456</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="J42" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="E42" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="G42" s="2" t="s">
+      <c r="K42" s="3" t="s">
         <v>458</v>
       </c>
-      <c r="H42" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="I42" s="2" t="s">
+      <c r="L42" s="3" t="s">
         <v>459</v>
       </c>
-      <c r="J42" s="2" t="s">
+      <c r="M42" s="3" t="s">
         <v>460</v>
       </c>
-      <c r="K42" s="2" t="s">
+      <c r="N42" s="5" t="s">
         <v>461</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="N42" s="5" t="s">
-        <v>464</v>
       </c>
       <c r="O42" s="4"/>
       <c r="P42" s="4"/>
@@ -5846,46 +5860,46 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="E43" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="G43" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="H43" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="I43" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="D43" s="2" t="s">
+      <c r="J43" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="E43" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="G43" s="2" t="s">
+      <c r="K43" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="H43" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="I43" s="2" t="s">
+      <c r="L43" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="J43" s="2" t="s">
+      <c r="M43" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="K43" s="2" t="s">
+      <c r="N43" s="5" t="s">
         <v>472</v>
-      </c>
-      <c r="L43" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="M43" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="N43" s="5" t="s">
-        <v>475</v>
       </c>
       <c r="O43" s="4"/>
       <c r="P43" s="4"/>
@@ -5904,46 +5918,46 @@
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="E44" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="H44" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="I44" s="2" t="s">
         <v>478</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="J44" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="E44" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="G44" s="2" t="s">
+      <c r="K44" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="H44" s="2" t="s">
-        <v>480</v>
-      </c>
-      <c r="I44" s="2" t="s">
+      <c r="L44" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="J44" s="2" t="s">
+      <c r="M44" s="2" t="s">
         <v>482</v>
       </c>
-      <c r="K44" s="2" t="s">
+      <c r="N44" s="5" t="s">
         <v>483</v>
-      </c>
-      <c r="L44" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="N44" s="5" t="s">
-        <v>486</v>
       </c>
       <c r="O44" s="4"/>
       <c r="P44" s="4"/>
@@ -5961,105 +5975,105 @@
       <c r="AB44" s="4"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="16" t="s">
+      <c r="A45" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>487</v>
       </c>
-      <c r="B45" s="17" t="s">
+      <c r="E45" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="G45" s="2" t="s">
         <v>488</v>
       </c>
-      <c r="C45" s="17" t="s">
+      <c r="H45" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="D45" s="17" t="s">
+      <c r="J45" s="2" t="s">
         <v>490</v>
       </c>
-      <c r="E45" s="17" t="s">
+      <c r="K45" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="F45" s="17" t="s">
-        <v>488</v>
-      </c>
-      <c r="G45" s="17" t="s">
+      <c r="L45" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="H45" s="17" t="s">
-        <v>492</v>
-      </c>
-      <c r="I45" s="17" t="s">
+      <c r="M45" s="2" t="s">
         <v>493</v>
       </c>
-      <c r="J45" s="17" t="s">
+      <c r="N45" s="5" t="s">
         <v>494</v>
       </c>
-      <c r="K45" s="18" t="s">
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
+      <c r="Q45" s="4"/>
+      <c r="R45" s="4"/>
+      <c r="S45" s="4"/>
+      <c r="T45" s="4"/>
+      <c r="U45" s="4"/>
+      <c r="V45" s="4"/>
+      <c r="W45" s="4"/>
+      <c r="X45" s="4"/>
+      <c r="Y45" s="4"/>
+      <c r="Z45" s="4"/>
+      <c r="AA45" s="4"/>
+      <c r="AB45" s="4"/>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="16" t="s">
         <v>495</v>
       </c>
-      <c r="L45" s="17" t="s">
+      <c r="B46" s="17" t="s">
         <v>496</v>
       </c>
-      <c r="M45" s="17" t="s">
+      <c r="C46" s="17" t="s">
         <v>497</v>
       </c>
-      <c r="N45" s="5" t="s">
+      <c r="D46" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="O45" s="19"/>
-      <c r="P45" s="19"/>
-      <c r="Q45" s="19"/>
-      <c r="R45" s="19"/>
-      <c r="S45" s="19"/>
-      <c r="T45" s="19"/>
-      <c r="U45" s="19"/>
-      <c r="V45" s="19"/>
-      <c r="W45" s="19"/>
-      <c r="X45" s="19"/>
-      <c r="Y45" s="19"/>
-      <c r="Z45" s="19"/>
-      <c r="AA45" s="19"/>
-      <c r="AB45" s="19"/>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="20" t="s">
+      <c r="E46" s="17" t="s">
         <v>499</v>
       </c>
-      <c r="B46" s="21" t="s">
+      <c r="F46" s="17" t="s">
+        <v>496</v>
+      </c>
+      <c r="G46" s="17" t="s">
         <v>500</v>
       </c>
-      <c r="C46" s="21" t="s">
+      <c r="H46" s="17" t="s">
+        <v>500</v>
+      </c>
+      <c r="I46" s="17" t="s">
         <v>501</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="J46" s="17" t="s">
         <v>502</v>
       </c>
-      <c r="E46" s="21" t="s">
+      <c r="K46" s="18" t="s">
         <v>503</v>
       </c>
-      <c r="F46" s="21" t="s">
-        <v>500</v>
-      </c>
-      <c r="G46" s="21" t="s">
+      <c r="L46" s="17" t="s">
         <v>504</v>
       </c>
-      <c r="H46" s="21" t="s">
-        <v>504</v>
-      </c>
-      <c r="I46" s="21" t="s">
+      <c r="M46" s="17" t="s">
         <v>505</v>
       </c>
-      <c r="J46" s="21" t="s">
+      <c r="N46" s="5" t="s">
         <v>506</v>
-      </c>
-      <c r="K46" s="18" t="s">
-        <v>507</v>
-      </c>
-      <c r="L46" s="21" t="s">
-        <v>508</v>
-      </c>
-      <c r="M46" s="21" t="s">
-        <v>509</v>
-      </c>
-      <c r="N46" s="5" t="s">
-        <v>510</v>
       </c>
       <c r="O46" s="19"/>
       <c r="P46" s="19"/>
@@ -6077,47 +6091,47 @@
       <c r="AB46" s="19"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="16" t="s">
+      <c r="A47" s="20" t="s">
+        <v>507</v>
+      </c>
+      <c r="B47" s="21" t="s">
+        <v>508</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>509</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>510</v>
+      </c>
+      <c r="E47" s="21" t="s">
         <v>511</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="F47" s="21" t="s">
+        <v>508</v>
+      </c>
+      <c r="G47" s="21" t="s">
         <v>512</v>
       </c>
-      <c r="C47" s="17" t="s">
+      <c r="H47" s="21" t="s">
+        <v>512</v>
+      </c>
+      <c r="I47" s="21" t="s">
         <v>513</v>
       </c>
-      <c r="D47" s="17" t="s">
+      <c r="J47" s="21" t="s">
         <v>514</v>
       </c>
-      <c r="E47" s="17" t="s">
+      <c r="K47" s="18" t="s">
         <v>515</v>
       </c>
-      <c r="F47" s="17" t="s">
-        <v>512</v>
-      </c>
-      <c r="G47" s="17" t="s">
+      <c r="L47" s="21" t="s">
         <v>516</v>
       </c>
-      <c r="H47" s="17" t="s">
-        <v>516</v>
-      </c>
-      <c r="I47" s="17" t="s">
+      <c r="M47" s="21" t="s">
         <v>517</v>
       </c>
-      <c r="J47" s="17" t="s">
+      <c r="N47" s="5" t="s">
         <v>518</v>
-      </c>
-      <c r="K47" s="18" t="s">
-        <v>519</v>
-      </c>
-      <c r="L47" s="17" t="s">
-        <v>520</v>
-      </c>
-      <c r="M47" s="17" t="s">
-        <v>521</v>
-      </c>
-      <c r="N47" s="5" t="s">
-        <v>522</v>
       </c>
       <c r="O47" s="19"/>
       <c r="P47" s="19"/>
@@ -6135,163 +6149,163 @@
       <c r="AB47" s="19"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="22" t="s">
+      <c r="A48" s="16" t="s">
+        <v>519</v>
+      </c>
+      <c r="B48" s="17" t="s">
+        <v>520</v>
+      </c>
+      <c r="C48" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="D48" s="17" t="s">
+        <v>522</v>
+      </c>
+      <c r="E48" s="17" t="s">
         <v>523</v>
       </c>
-      <c r="B48" s="23" t="s">
+      <c r="F48" s="17" t="s">
+        <v>520</v>
+      </c>
+      <c r="G48" s="17" t="s">
         <v>524</v>
       </c>
-      <c r="C48" s="23" t="s">
+      <c r="H48" s="17" t="s">
+        <v>524</v>
+      </c>
+      <c r="I48" s="17" t="s">
         <v>525</v>
       </c>
-      <c r="D48" s="23" t="s">
+      <c r="J48" s="17" t="s">
         <v>526</v>
       </c>
-      <c r="E48" s="23" t="s">
-        <v>524</v>
-      </c>
-      <c r="F48" s="23" t="s">
-        <v>524</v>
-      </c>
-      <c r="G48" s="23" t="s">
+      <c r="K48" s="18" t="s">
         <v>527</v>
       </c>
-      <c r="H48" s="23" t="s">
-        <v>527</v>
-      </c>
-      <c r="I48" s="23" t="s">
+      <c r="L48" s="17" t="s">
         <v>528</v>
       </c>
-      <c r="J48" s="23" t="s">
+      <c r="M48" s="17" t="s">
         <v>529</v>
       </c>
-      <c r="K48" s="23" t="s">
+      <c r="N48" s="5" t="s">
         <v>530</v>
       </c>
-      <c r="L48" s="23" t="s">
+      <c r="O48" s="19"/>
+      <c r="P48" s="19"/>
+      <c r="Q48" s="19"/>
+      <c r="R48" s="19"/>
+      <c r="S48" s="19"/>
+      <c r="T48" s="19"/>
+      <c r="U48" s="19"/>
+      <c r="V48" s="19"/>
+      <c r="W48" s="19"/>
+      <c r="X48" s="19"/>
+      <c r="Y48" s="19"/>
+      <c r="Z48" s="19"/>
+      <c r="AA48" s="19"/>
+      <c r="AB48" s="19"/>
+    </row>
+    <row r="49" ht="15.75" customHeight="1">
+      <c r="A49" s="22" t="s">
         <v>531</v>
       </c>
-      <c r="M48" s="23" t="s">
+      <c r="B49" s="23" t="s">
         <v>532</v>
       </c>
-      <c r="N48" s="5" t="s">
+      <c r="C49" s="23" t="s">
         <v>533</v>
       </c>
-      <c r="O48" s="24"/>
-      <c r="P48" s="24"/>
-      <c r="Q48" s="24"/>
-      <c r="R48" s="24"/>
-      <c r="S48" s="24"/>
-      <c r="T48" s="24"/>
-      <c r="U48" s="24"/>
-      <c r="V48" s="24"/>
-      <c r="W48" s="24"/>
-      <c r="X48" s="24"/>
-      <c r="Y48" s="24"/>
-      <c r="Z48" s="24"/>
-      <c r="AA48" s="24"/>
-      <c r="AB48" s="24"/>
-    </row>
-    <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="1" t="s">
+      <c r="D49" s="23" t="s">
         <v>534</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I49" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="L49" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M49" s="2" t="s">
-        <v>39</v>
+      <c r="E49" s="23" t="s">
+        <v>532</v>
+      </c>
+      <c r="F49" s="23" t="s">
+        <v>532</v>
+      </c>
+      <c r="G49" s="23" t="s">
+        <v>535</v>
+      </c>
+      <c r="H49" s="23" t="s">
+        <v>535</v>
+      </c>
+      <c r="I49" s="23" t="s">
+        <v>536</v>
+      </c>
+      <c r="J49" s="23" t="s">
+        <v>537</v>
+      </c>
+      <c r="K49" s="23" t="s">
+        <v>538</v>
+      </c>
+      <c r="L49" s="23" t="s">
+        <v>539</v>
+      </c>
+      <c r="M49" s="23" t="s">
+        <v>540</v>
       </c>
       <c r="N49" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="O49" s="4"/>
-      <c r="P49" s="4"/>
-      <c r="Q49" s="4"/>
-      <c r="R49" s="4"/>
-      <c r="S49" s="4"/>
-      <c r="T49" s="4"/>
-      <c r="U49" s="4"/>
-      <c r="V49" s="4"/>
-      <c r="W49" s="4"/>
-      <c r="X49" s="4"/>
-      <c r="Y49" s="4"/>
-      <c r="Z49" s="4"/>
-      <c r="AA49" s="4"/>
-      <c r="AB49" s="4"/>
+        <v>541</v>
+      </c>
+      <c r="O49" s="24"/>
+      <c r="P49" s="24"/>
+      <c r="Q49" s="24"/>
+      <c r="R49" s="24"/>
+      <c r="S49" s="24"/>
+      <c r="T49" s="24"/>
+      <c r="U49" s="24"/>
+      <c r="V49" s="24"/>
+      <c r="W49" s="24"/>
+      <c r="X49" s="24"/>
+      <c r="Y49" s="24"/>
+      <c r="Z49" s="24"/>
+      <c r="AA49" s="24"/>
+      <c r="AB49" s="24"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="1" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>536</v>
+        <v>32</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>537</v>
+        <v>33</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>538</v>
+        <v>34</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>536</v>
+        <v>32</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>536</v>
+        <v>32</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>539</v>
+        <v>32</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>539</v>
+        <v>32</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>540</v>
+        <v>35</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>541</v>
+        <v>36</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>542</v>
+        <v>37</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>543</v>
+        <v>38</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>544</v>
+        <v>39</v>
       </c>
       <c r="N50" s="5" t="s">
-        <v>545</v>
+        <v>40</v>
       </c>
       <c r="O50" s="4"/>
       <c r="P50" s="4"/>
@@ -6310,46 +6324,46 @@
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>546</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="E51" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="G51" s="2" t="s">
         <v>547</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="H51" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="I51" s="2" t="s">
         <v>548</v>
       </c>
-      <c r="D51" s="2" t="s">
+      <c r="J51" s="2" t="s">
         <v>549</v>
       </c>
-      <c r="E51" s="2" t="s">
-        <v>547</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>547</v>
-      </c>
-      <c r="G51" s="2" t="s">
+      <c r="K51" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="H51" s="2" t="s">
-        <v>550</v>
-      </c>
-      <c r="I51" s="2" t="s">
+      <c r="L51" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="J51" s="2" t="s">
+      <c r="M51" s="2" t="s">
         <v>552</v>
       </c>
-      <c r="K51" s="2" t="s">
+      <c r="N51" s="5" t="s">
         <v>553</v>
-      </c>
-      <c r="L51" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="M51" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="N51" s="5" t="s">
-        <v>554</v>
       </c>
       <c r="O51" s="4"/>
       <c r="P51" s="4"/>
@@ -6368,46 +6382,46 @@
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="C52" s="2" t="s">
         <v>556</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="D52" s="2" t="s">
         <v>557</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="E52" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="G52" s="2" t="s">
         <v>558</v>
       </c>
-      <c r="E52" s="2" t="s">
-        <v>556</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>556</v>
-      </c>
-      <c r="G52" s="2" t="s">
+      <c r="H52" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="I52" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="H52" s="2" t="s">
-        <v>559</v>
-      </c>
-      <c r="I52" s="2" t="s">
+      <c r="J52" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="J52" s="2" t="s">
+      <c r="K52" s="2" t="s">
         <v>561</v>
       </c>
-      <c r="K52" s="2" t="s">
+      <c r="L52" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M52" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="N52" s="5" t="s">
         <v>562</v>
-      </c>
-      <c r="L52" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="M52" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="N52" s="5" t="s">
-        <v>565</v>
       </c>
       <c r="O52" s="4"/>
       <c r="P52" s="4"/>
@@ -6426,46 +6440,46 @@
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>566</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="E53" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="G53" s="2" t="s">
         <v>567</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="H53" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="I53" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="D53" s="2" t="s">
+      <c r="J53" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="E53" s="2" t="s">
-        <v>567</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>567</v>
-      </c>
-      <c r="G53" s="2" t="s">
+      <c r="K53" s="2" t="s">
         <v>570</v>
       </c>
-      <c r="H53" s="2" t="s">
+      <c r="L53" s="2" t="s">
         <v>571</v>
       </c>
-      <c r="I53" s="2" t="s">
+      <c r="M53" s="2" t="s">
         <v>572</v>
       </c>
-      <c r="J53" s="2" t="s">
+      <c r="N53" s="5" t="s">
         <v>573</v>
-      </c>
-      <c r="K53" s="2" t="s">
-        <v>574</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>575</v>
-      </c>
-      <c r="M53" s="2" t="s">
-        <v>576</v>
-      </c>
-      <c r="N53" s="5" t="s">
-        <v>577</v>
       </c>
       <c r="O53" s="4"/>
       <c r="P53" s="4"/>
@@ -6484,46 +6498,46 @@
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="G54" s="2" t="s">
         <v>578</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="H54" s="2" t="s">
         <v>579</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="I54" s="2" t="s">
         <v>580</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="J54" s="2" t="s">
         <v>581</v>
       </c>
-      <c r="E54" s="2" t="s">
-        <v>579</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>579</v>
-      </c>
-      <c r="G54" s="2" t="s">
+      <c r="K54" s="2" t="s">
         <v>582</v>
       </c>
-      <c r="H54" s="2" t="s">
-        <v>582</v>
-      </c>
-      <c r="I54" s="2" t="s">
+      <c r="L54" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="J54" s="2" t="s">
+      <c r="M54" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="K54" s="2" t="s">
+      <c r="N54" s="5" t="s">
         <v>585</v>
-      </c>
-      <c r="L54" s="2" t="s">
-        <v>586</v>
-      </c>
-      <c r="M54" s="3" t="s">
-        <v>587</v>
-      </c>
-      <c r="N54" s="5" t="s">
-        <v>588</v>
       </c>
       <c r="O54" s="4"/>
       <c r="P54" s="4"/>
@@ -6542,46 +6556,46 @@
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>589</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="E55" s="2" t="s">
-        <v>42</v>
+        <v>587</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>42</v>
+        <v>587</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>45</v>
+        <v>590</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>45</v>
+        <v>590</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>45</v>
+        <v>591</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>46</v>
+        <v>592</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>47</v>
+        <v>593</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="M55" s="2" t="s">
-        <v>49</v>
+        <v>594</v>
+      </c>
+      <c r="M55" s="3" t="s">
+        <v>595</v>
       </c>
       <c r="N55" s="5" t="s">
-        <v>50</v>
+        <v>596</v>
       </c>
       <c r="O55" s="4"/>
       <c r="P55" s="4"/>
@@ -6600,46 +6614,46 @@
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="1" t="s">
-        <v>590</v>
+        <v>597</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>591</v>
+        <v>42</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>592</v>
+        <v>43</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>593</v>
+        <v>44</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>591</v>
+        <v>42</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>591</v>
+        <v>42</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>594</v>
+        <v>45</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>594</v>
+        <v>45</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>595</v>
-      </c>
-      <c r="J56" s="3" t="s">
-        <v>596</v>
+        <v>45</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>597</v>
+        <v>47</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>598</v>
+        <v>48</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>599</v>
+        <v>49</v>
       </c>
       <c r="N56" s="5" t="s">
-        <v>600</v>
+        <v>50</v>
       </c>
       <c r="O56" s="4"/>
       <c r="P56" s="4"/>
@@ -6657,47 +6671,47 @@
       <c r="AB56" s="4"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="25" t="s">
+      <c r="A57" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>601</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="E57" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="G57" s="2" t="s">
         <v>602</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="H57" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="I57" s="2" t="s">
         <v>603</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="J57" s="3" t="s">
         <v>604</v>
       </c>
-      <c r="E57" s="2" t="s">
-        <v>602</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>602</v>
-      </c>
-      <c r="G57" s="2" t="s">
+      <c r="K57" s="2" t="s">
         <v>605</v>
       </c>
-      <c r="H57" s="2" t="s">
-        <v>605</v>
-      </c>
-      <c r="I57" s="2" t="s">
+      <c r="L57" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="J57" s="2" t="s">
+      <c r="M57" s="2" t="s">
         <v>607</v>
       </c>
-      <c r="K57" s="2" t="s">
+      <c r="N57" s="5" t="s">
         <v>608</v>
-      </c>
-      <c r="L57" s="2" t="s">
-        <v>609</v>
-      </c>
-      <c r="M57" s="2" t="s">
-        <v>610</v>
-      </c>
-      <c r="N57" s="5" t="s">
-        <v>611</v>
       </c>
       <c r="O57" s="4"/>
       <c r="P57" s="4"/>
@@ -6715,47 +6729,47 @@
       <c r="AB57" s="4"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="1" t="s">
+      <c r="A58" s="25" t="s">
+        <v>609</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>612</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="E58" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="G58" s="2" t="s">
         <v>613</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="H58" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="I58" s="2" t="s">
         <v>614</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="J58" s="2" t="s">
         <v>615</v>
       </c>
-      <c r="E58" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="G58" s="2" t="s">
+      <c r="K58" s="2" t="s">
         <v>616</v>
       </c>
-      <c r="H58" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="I58" s="2" t="s">
+      <c r="L58" s="2" t="s">
         <v>617</v>
       </c>
-      <c r="J58" s="2" t="s">
+      <c r="M58" s="2" t="s">
         <v>618</v>
       </c>
-      <c r="K58" s="2" t="s">
+      <c r="N58" s="5" t="s">
         <v>619</v>
-      </c>
-      <c r="L58" s="2" t="s">
-        <v>620</v>
-      </c>
-      <c r="M58" s="2" t="s">
-        <v>621</v>
-      </c>
-      <c r="N58" s="5" t="s">
-        <v>622</v>
       </c>
       <c r="O58" s="4"/>
       <c r="P58" s="4"/>
@@ -6774,46 +6788,46 @@
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="1" t="s">
+        <v>620</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>623</v>
       </c>
-      <c r="B59" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>293</v>
-      </c>
       <c r="E59" s="2" t="s">
-        <v>291</v>
+        <v>621</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>291</v>
+        <v>621</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>294</v>
+        <v>624</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>294</v>
+        <v>624</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>296</v>
+        <v>626</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>297</v>
+        <v>627</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>298</v>
+        <v>628</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>299</v>
+        <v>629</v>
       </c>
       <c r="N59" s="5" t="s">
-        <v>300</v>
+        <v>630</v>
       </c>
       <c r="O59" s="4"/>
       <c r="P59" s="4"/>
@@ -6832,46 +6846,46 @@
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="1" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>466</v>
+        <v>299</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>467</v>
+        <v>300</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>468</v>
+        <v>301</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>466</v>
+        <v>299</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>466</v>
+        <v>299</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>469</v>
+        <v>302</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>469</v>
+        <v>302</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>470</v>
+        <v>632</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>471</v>
+        <v>304</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>472</v>
+        <v>305</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>473</v>
+        <v>306</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>474</v>
+        <v>307</v>
       </c>
       <c r="N60" s="5" t="s">
-        <v>475</v>
+        <v>308</v>
       </c>
       <c r="O60" s="4"/>
       <c r="P60" s="4"/>
@@ -6890,46 +6904,46 @@
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="1" t="s">
-        <v>626</v>
+        <v>633</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>627</v>
+        <v>474</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>628</v>
+        <v>475</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>629</v>
+        <v>476</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>627</v>
+        <v>474</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>627</v>
+        <v>474</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>630</v>
+        <v>477</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>630</v>
+        <v>477</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>631</v>
+        <v>478</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>632</v>
+        <v>479</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>633</v>
+        <v>480</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>634</v>
+        <v>481</v>
       </c>
       <c r="M61" s="2" t="s">
-        <v>634</v>
+        <v>482</v>
       </c>
       <c r="N61" s="5" t="s">
-        <v>635</v>
+        <v>483</v>
       </c>
       <c r="O61" s="4"/>
       <c r="P61" s="4"/>
@@ -6947,47 +6961,47 @@
       <c r="AB61" s="4"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="25" t="s">
+      <c r="A62" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>636</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="D62" s="2" t="s">
         <v>637</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="E62" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="G62" s="2" t="s">
         <v>638</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="H62" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="I62" s="2" t="s">
         <v>639</v>
       </c>
-      <c r="E62" s="2" t="s">
+      <c r="J62" s="2" t="s">
         <v>640</v>
       </c>
-      <c r="F62" s="2" t="s">
-        <v>637</v>
-      </c>
-      <c r="G62" s="2" t="s">
+      <c r="K62" s="2" t="s">
         <v>641</v>
       </c>
-      <c r="H62" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="I62" s="2" t="s">
+      <c r="L62" s="2" t="s">
         <v>642</v>
       </c>
-      <c r="J62" s="2" t="s">
+      <c r="M62" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="N62" s="5" t="s">
         <v>643</v>
-      </c>
-      <c r="K62" s="2" t="s">
-        <v>644</v>
-      </c>
-      <c r="L62" s="2" t="s">
-        <v>645</v>
-      </c>
-      <c r="M62" s="2" t="s">
-        <v>646</v>
-      </c>
-      <c r="N62" s="5" t="s">
-        <v>647</v>
       </c>
       <c r="O62" s="4"/>
       <c r="P62" s="4"/>
@@ -7005,337 +7019,337 @@
       <c r="AB62" s="4"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="22" t="s">
+      <c r="A63" s="25" t="s">
+        <v>644</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="E63" s="2" t="s">
         <v>648</v>
       </c>
-      <c r="B63" s="23" t="s">
+      <c r="F63" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="G63" s="2" t="s">
         <v>649</v>
       </c>
-      <c r="C63" s="23" t="s">
+      <c r="H63" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="I63" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="D63" s="23" t="s">
+      <c r="J63" s="2" t="s">
         <v>651</v>
       </c>
-      <c r="E63" s="23" t="s">
-        <v>649</v>
-      </c>
-      <c r="F63" s="23" t="s">
-        <v>649</v>
-      </c>
-      <c r="G63" s="23" t="s">
+      <c r="K63" s="2" t="s">
         <v>652</v>
       </c>
-      <c r="H63" s="23" t="s">
-        <v>652</v>
-      </c>
-      <c r="I63" s="23" t="s">
+      <c r="L63" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="J63" s="23" t="s">
+      <c r="M63" s="2" t="s">
         <v>654</v>
       </c>
-      <c r="K63" s="23" t="s">
+      <c r="N63" s="5" t="s">
         <v>655</v>
       </c>
-      <c r="L63" s="23" t="s">
+      <c r="O63" s="4"/>
+      <c r="P63" s="4"/>
+      <c r="Q63" s="4"/>
+      <c r="R63" s="4"/>
+      <c r="S63" s="4"/>
+      <c r="T63" s="4"/>
+      <c r="U63" s="4"/>
+      <c r="V63" s="4"/>
+      <c r="W63" s="4"/>
+      <c r="X63" s="4"/>
+      <c r="Y63" s="4"/>
+      <c r="Z63" s="4"/>
+      <c r="AA63" s="4"/>
+      <c r="AB63" s="4"/>
+    </row>
+    <row r="64" ht="15.75" customHeight="1">
+      <c r="A64" s="22" t="s">
         <v>656</v>
       </c>
-      <c r="M63" s="23" t="s">
+      <c r="B64" s="23" t="s">
         <v>657</v>
       </c>
-      <c r="N63" s="5" t="s">
+      <c r="C64" s="23" t="s">
         <v>658</v>
       </c>
-      <c r="O63" s="24"/>
-      <c r="P63" s="24"/>
-      <c r="Q63" s="24"/>
-      <c r="R63" s="24"/>
-      <c r="S63" s="24"/>
-      <c r="T63" s="24"/>
-      <c r="U63" s="24"/>
-      <c r="V63" s="24"/>
-      <c r="W63" s="24"/>
-      <c r="X63" s="24"/>
-      <c r="Y63" s="24"/>
-      <c r="Z63" s="24"/>
-      <c r="AA63" s="24"/>
-      <c r="AB63" s="24"/>
-    </row>
-    <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="26" t="s">
+      <c r="D64" s="23" t="s">
         <v>659</v>
       </c>
-      <c r="B64" s="27" t="s">
+      <c r="E64" s="23" t="s">
+        <v>657</v>
+      </c>
+      <c r="F64" s="23" t="s">
+        <v>657</v>
+      </c>
+      <c r="G64" s="23" t="s">
         <v>660</v>
       </c>
-      <c r="C64" s="27" t="s">
+      <c r="H64" s="23" t="s">
+        <v>660</v>
+      </c>
+      <c r="I64" s="23" t="s">
         <v>661</v>
       </c>
-      <c r="D64" s="27" t="s">
+      <c r="J64" s="23" t="s">
         <v>662</v>
       </c>
-      <c r="E64" s="27" t="s">
+      <c r="K64" s="23" t="s">
         <v>663</v>
       </c>
-      <c r="F64" s="27" t="s">
-        <v>663</v>
-      </c>
-      <c r="G64" s="27" t="s">
+      <c r="L64" s="23" t="s">
         <v>664</v>
       </c>
-      <c r="H64" s="27" t="s">
-        <v>664</v>
-      </c>
-      <c r="I64" s="27" t="s">
+      <c r="M64" s="23" t="s">
         <v>665</v>
       </c>
-      <c r="J64" s="27" t="s">
+      <c r="N64" s="5" t="s">
         <v>666</v>
       </c>
-      <c r="K64" s="28" t="s">
+      <c r="O64" s="24"/>
+      <c r="P64" s="24"/>
+      <c r="Q64" s="24"/>
+      <c r="R64" s="24"/>
+      <c r="S64" s="24"/>
+      <c r="T64" s="24"/>
+      <c r="U64" s="24"/>
+      <c r="V64" s="24"/>
+      <c r="W64" s="24"/>
+      <c r="X64" s="24"/>
+      <c r="Y64" s="24"/>
+      <c r="Z64" s="24"/>
+      <c r="AA64" s="24"/>
+      <c r="AB64" s="24"/>
+    </row>
+    <row r="65" ht="15.75" customHeight="1">
+      <c r="A65" s="26" t="s">
         <v>667</v>
       </c>
-      <c r="L64" s="27" t="s">
+      <c r="B65" s="27" t="s">
         <v>668</v>
       </c>
-      <c r="M64" s="27" t="s">
+      <c r="C65" s="27" t="s">
         <v>669</v>
       </c>
-      <c r="N64" s="5" t="s">
+      <c r="D65" s="27" t="s">
         <v>670</v>
       </c>
-      <c r="O64" s="29"/>
-      <c r="P64" s="29"/>
-      <c r="Q64" s="29"/>
-      <c r="R64" s="29"/>
-      <c r="S64" s="29"/>
-      <c r="T64" s="29"/>
-      <c r="U64" s="29"/>
-      <c r="V64" s="29"/>
-      <c r="W64" s="29"/>
-      <c r="X64" s="29"/>
-      <c r="Y64" s="29"/>
-      <c r="Z64" s="29"/>
-      <c r="AA64" s="29"/>
-      <c r="AB64" s="29"/>
-    </row>
-    <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="9" t="s">
+      <c r="E65" s="27" t="s">
         <v>671</v>
       </c>
-      <c r="B65" s="3" t="s">
+      <c r="F65" s="27" t="s">
+        <v>671</v>
+      </c>
+      <c r="G65" s="27" t="s">
         <v>672</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="H65" s="27" t="s">
+        <v>672</v>
+      </c>
+      <c r="I65" s="27" t="s">
         <v>673</v>
       </c>
-      <c r="D65" s="3" t="s">
+      <c r="J65" s="27" t="s">
         <v>674</v>
       </c>
-      <c r="E65" s="11" t="s">
-        <v>672</v>
-      </c>
-      <c r="F65" s="3" t="s">
+      <c r="K65" s="28" t="s">
         <v>675</v>
       </c>
-      <c r="G65" s="3" t="s">
+      <c r="L65" s="27" t="s">
         <v>676</v>
       </c>
-      <c r="H65" s="3" t="s">
-        <v>676</v>
-      </c>
-      <c r="I65" s="3" t="s">
+      <c r="M65" s="27" t="s">
         <v>677</v>
       </c>
-      <c r="J65" s="3" t="s">
+      <c r="N65" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="K65" s="3" t="s">
-        <v>678</v>
-      </c>
-      <c r="L65" s="3" t="s">
+      <c r="O65" s="29"/>
+      <c r="P65" s="29"/>
+      <c r="Q65" s="29"/>
+      <c r="R65" s="29"/>
+      <c r="S65" s="29"/>
+      <c r="T65" s="29"/>
+      <c r="U65" s="29"/>
+      <c r="V65" s="29"/>
+      <c r="W65" s="29"/>
+      <c r="X65" s="29"/>
+      <c r="Y65" s="29"/>
+      <c r="Z65" s="29"/>
+      <c r="AA65" s="29"/>
+      <c r="AB65" s="29"/>
+    </row>
+    <row r="66" ht="15.75" customHeight="1">
+      <c r="A66" s="9" t="s">
         <v>679</v>
       </c>
-      <c r="M65" s="3" t="s">
+      <c r="B66" s="3" t="s">
         <v>680</v>
       </c>
-      <c r="N65" s="3" t="s">
+      <c r="C66" s="3" t="s">
         <v>681</v>
       </c>
-      <c r="O65" s="4"/>
-      <c r="P65" s="4"/>
-      <c r="Q65" s="4"/>
-      <c r="R65" s="4"/>
-      <c r="S65" s="4"/>
-      <c r="T65" s="4"/>
-      <c r="U65" s="4"/>
-      <c r="V65" s="4"/>
-      <c r="W65" s="4"/>
-      <c r="X65" s="4"/>
-      <c r="Y65" s="4"/>
-      <c r="Z65" s="4"/>
-      <c r="AA65" s="4"/>
-      <c r="AB65" s="4"/>
-    </row>
-    <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="14" t="s">
+      <c r="D66" s="3" t="s">
         <v>682</v>
       </c>
-      <c r="B66" s="15" t="s">
+      <c r="E66" s="11" t="s">
+        <v>680</v>
+      </c>
+      <c r="F66" s="3" t="s">
         <v>683</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="G66" s="3" t="s">
         <v>684</v>
       </c>
-      <c r="D66" s="3" t="s">
+      <c r="H66" s="3" t="s">
+        <v>684</v>
+      </c>
+      <c r="I66" s="3" t="s">
         <v>685</v>
       </c>
-      <c r="E66" s="11" t="s">
-        <v>683</v>
-      </c>
-      <c r="F66" s="3" t="s">
+      <c r="J66" s="3" t="s">
         <v>686</v>
       </c>
-      <c r="G66" s="3" t="s">
+      <c r="K66" s="3" t="s">
+        <v>686</v>
+      </c>
+      <c r="L66" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="H66" s="3" t="s">
-        <v>687</v>
-      </c>
-      <c r="I66" s="3" t="s">
+      <c r="M66" s="3" t="s">
         <v>688</v>
       </c>
-      <c r="J66" s="3" t="s">
+      <c r="N66" s="3" t="s">
         <v>689</v>
       </c>
-      <c r="K66" s="3" t="s">
-        <v>689</v>
-      </c>
-      <c r="L66" s="3" t="s">
+      <c r="O66" s="4"/>
+      <c r="P66" s="4"/>
+      <c r="Q66" s="4"/>
+      <c r="R66" s="4"/>
+      <c r="S66" s="4"/>
+      <c r="T66" s="4"/>
+      <c r="U66" s="4"/>
+      <c r="V66" s="4"/>
+      <c r="W66" s="4"/>
+      <c r="X66" s="4"/>
+      <c r="Y66" s="4"/>
+      <c r="Z66" s="4"/>
+      <c r="AA66" s="4"/>
+      <c r="AB66" s="4"/>
+    </row>
+    <row r="67" ht="15.75" customHeight="1">
+      <c r="A67" s="14" t="s">
         <v>690</v>
       </c>
-      <c r="M66" s="3" t="s">
+      <c r="B67" s="15" t="s">
         <v>691</v>
       </c>
-      <c r="N66" s="3" t="s">
+      <c r="C67" s="3" t="s">
         <v>692</v>
       </c>
-      <c r="O66" s="30"/>
-      <c r="P66" s="30"/>
-      <c r="Q66" s="30"/>
-      <c r="R66" s="30"/>
-      <c r="S66" s="30"/>
-      <c r="T66" s="30"/>
-      <c r="U66" s="30"/>
-      <c r="V66" s="30"/>
-      <c r="W66" s="30"/>
-      <c r="X66" s="30"/>
-      <c r="Y66" s="30"/>
-      <c r="Z66" s="30"/>
-      <c r="AA66" s="30"/>
-      <c r="AB66" s="30"/>
-    </row>
-    <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="9" t="s">
+      <c r="D67" s="3" t="s">
         <v>693</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="E67" s="11" t="s">
+        <v>691</v>
+      </c>
+      <c r="F67" s="3" t="s">
         <v>694</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="G67" s="3" t="s">
         <v>695</v>
       </c>
-      <c r="D67" s="2" t="s">
+      <c r="H67" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="I67" s="3" t="s">
         <v>696</v>
       </c>
-      <c r="E67" s="2" t="s">
-        <v>694</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>694</v>
-      </c>
-      <c r="G67" s="3" t="s">
+      <c r="J67" s="3" t="s">
         <v>697</v>
       </c>
-      <c r="H67" s="3" t="s">
+      <c r="K67" s="3" t="s">
         <v>697</v>
       </c>
-      <c r="I67" s="3" t="s">
+      <c r="L67" s="3" t="s">
         <v>698</v>
       </c>
-      <c r="J67" s="2" t="s">
+      <c r="M67" s="3" t="s">
         <v>699</v>
       </c>
-      <c r="K67" s="3" t="s">
+      <c r="N67" s="3" t="s">
         <v>700</v>
       </c>
-      <c r="L67" s="2" t="s">
-        <v>701</v>
-      </c>
-      <c r="M67" s="2" t="s">
-        <v>702</v>
-      </c>
-      <c r="N67" s="5" t="s">
-        <v>703</v>
-      </c>
-      <c r="O67" s="4"/>
-      <c r="P67" s="4"/>
-      <c r="Q67" s="4"/>
-      <c r="R67" s="4"/>
-      <c r="S67" s="4"/>
-      <c r="T67" s="4"/>
-      <c r="U67" s="4"/>
-      <c r="V67" s="4"/>
-      <c r="W67" s="4"/>
-      <c r="X67" s="4"/>
-      <c r="Y67" s="4"/>
-      <c r="Z67" s="4"/>
-      <c r="AA67" s="4"/>
-      <c r="AB67" s="4"/>
+      <c r="O67" s="30"/>
+      <c r="P67" s="30"/>
+      <c r="Q67" s="30"/>
+      <c r="R67" s="30"/>
+      <c r="S67" s="30"/>
+      <c r="T67" s="30"/>
+      <c r="U67" s="30"/>
+      <c r="V67" s="30"/>
+      <c r="W67" s="30"/>
+      <c r="X67" s="30"/>
+      <c r="Y67" s="30"/>
+      <c r="Z67" s="30"/>
+      <c r="AA67" s="30"/>
+      <c r="AB67" s="30"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="9" t="s">
+        <v>701</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>704</v>
       </c>
-      <c r="B68" s="3" t="s">
+      <c r="E68" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="G68" s="3" t="s">
         <v>705</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="H68" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="I68" s="3" t="s">
         <v>706</v>
       </c>
-      <c r="D68" s="3" t="s">
+      <c r="J68" s="3" t="s">
         <v>707</v>
       </c>
-      <c r="E68" s="31" t="s">
+      <c r="K68" s="3" t="s">
         <v>708</v>
       </c>
-      <c r="F68" s="3" t="s">
+      <c r="L68" s="2" t="s">
         <v>709</v>
       </c>
-      <c r="G68" s="3" t="s">
+      <c r="M68" s="2" t="s">
         <v>710</v>
       </c>
-      <c r="H68" s="3" t="s">
-        <v>710</v>
-      </c>
-      <c r="I68" s="3" t="s">
+      <c r="N68" s="5" t="s">
         <v>711</v>
-      </c>
-      <c r="J68" s="3" t="s">
-        <v>712</v>
-      </c>
-      <c r="K68" s="3" t="s">
-        <v>713</v>
-      </c>
-      <c r="L68" s="3" t="s">
-        <v>714</v>
-      </c>
-      <c r="M68" s="3" t="s">
-        <v>715</v>
-      </c>
-      <c r="N68" s="5" t="s">
-        <v>716</v>
       </c>
       <c r="O68" s="4"/>
       <c r="P68" s="4"/>
@@ -7353,43 +7367,43 @@
       <c r="AB68" s="4"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="1" t="s">
+      <c r="A69" s="9" t="s">
+        <v>712</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>714</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="E69" s="31" t="s">
+        <v>716</v>
+      </c>
+      <c r="F69" s="3" t="s">
         <v>717</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="G69" s="3" t="s">
         <v>718</v>
       </c>
-      <c r="C69" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="D69" s="2" t="s">
+      <c r="H69" s="3" t="s">
+        <v>718</v>
+      </c>
+      <c r="I69" s="3" t="s">
         <v>719</v>
       </c>
-      <c r="E69" s="2" t="s">
-        <v>718</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>718</v>
-      </c>
-      <c r="G69" s="2" t="s">
+      <c r="J69" s="3" t="s">
         <v>720</v>
       </c>
-      <c r="H69" s="2" t="s">
-        <v>720</v>
-      </c>
-      <c r="I69" s="2" t="s">
+      <c r="K69" s="3" t="s">
         <v>721</v>
       </c>
-      <c r="J69" s="2" t="s">
-        <v>529</v>
-      </c>
-      <c r="K69" s="2" t="s">
-        <v>530</v>
-      </c>
-      <c r="L69" s="2" t="s">
+      <c r="L69" s="3" t="s">
         <v>722</v>
       </c>
-      <c r="M69" s="2" t="s">
+      <c r="M69" s="3" t="s">
         <v>723</v>
       </c>
       <c r="N69" s="5" t="s">
@@ -7415,43 +7429,43 @@
         <v>725</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>694</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>695</v>
+        <v>726</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>533</v>
       </c>
       <c r="D70" s="2" t="s">
+        <v>727</v>
+      </c>
+      <c r="E70" s="2" t="s">
         <v>726</v>
       </c>
-      <c r="E70" s="2" t="s">
-        <v>694</v>
-      </c>
       <c r="F70" s="2" t="s">
-        <v>694</v>
+        <v>726</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="I70" s="2" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="J70" s="2" t="s">
-        <v>699</v>
-      </c>
-      <c r="K70" s="3" t="s">
-        <v>700</v>
+        <v>537</v>
+      </c>
+      <c r="K70" s="2" t="s">
+        <v>538</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="M70" s="2" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="N70" s="5" t="s">
-        <v>703</v>
+        <v>732</v>
       </c>
       <c r="O70" s="4"/>
       <c r="P70" s="4"/>
@@ -7470,46 +7484,46 @@
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="1" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>731</v>
+        <v>702</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>703</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>54</v>
+        <v>734</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>52</v>
+        <v>702</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>52</v>
+        <v>702</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>55</v>
+        <v>735</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>55</v>
+        <v>735</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="J71" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="K71" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="L71" s="3" t="s">
-        <v>59</v>
+        <v>735</v>
+      </c>
+      <c r="J71" s="3" t="s">
+        <v>707</v>
+      </c>
+      <c r="K71" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L71" s="2" t="s">
+        <v>736</v>
       </c>
       <c r="M71" s="2" t="s">
-        <v>60</v>
+        <v>737</v>
       </c>
       <c r="N71" s="5" t="s">
-        <v>61</v>
+        <v>711</v>
       </c>
       <c r="O71" s="4"/>
       <c r="P71" s="4"/>
@@ -7528,46 +7542,46 @@
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="1" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>87</v>
+        <v>739</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>88</v>
+        <v>54</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>89</v>
+        <v>55</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>89</v>
+        <v>55</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>91</v>
+        <v>56</v>
       </c>
       <c r="J72" s="2" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="L72" s="2" t="s">
-        <v>733</v>
+        <v>58</v>
+      </c>
+      <c r="L72" s="3" t="s">
+        <v>59</v>
       </c>
       <c r="M72" s="2" t="s">
-        <v>734</v>
+        <v>60</v>
       </c>
       <c r="N72" s="5" t="s">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="O72" s="4"/>
       <c r="P72" s="4"/>
@@ -7586,46 +7600,46 @@
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="1" t="s">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>364</v>
+        <v>86</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>736</v>
+        <v>87</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>737</v>
+        <v>88</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>367</v>
+        <v>86</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>364</v>
+        <v>86</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>368</v>
+        <v>89</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="I73" s="3" t="s">
-        <v>738</v>
+        <v>89</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="J73" s="2" t="s">
-        <v>739</v>
+        <v>92</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="L73" s="3" t="s">
-        <v>372</v>
+        <v>93</v>
+      </c>
+      <c r="L73" s="2" t="s">
+        <v>741</v>
       </c>
       <c r="M73" s="2" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="N73" s="5" t="s">
-        <v>374</v>
+        <v>96</v>
       </c>
       <c r="O73" s="4"/>
       <c r="P73" s="4"/>
@@ -7644,46 +7658,46 @@
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="1" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="B74" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>745</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="G74" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="C74" s="2" t="s">
-        <v>742</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="E74" s="2" t="s">
+      <c r="H74" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>746</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="K74" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="F74" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="G74" s="2" t="s">
+      <c r="L74" s="3" t="s">
         <v>380</v>
       </c>
-      <c r="H74" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="I74" s="3" t="s">
-        <v>743</v>
-      </c>
-      <c r="J74" s="2" t="s">
+      <c r="M74" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="N74" s="5" t="s">
         <v>382</v>
-      </c>
-      <c r="K74" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="L74" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="M74" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="N74" s="5" t="s">
-        <v>386</v>
       </c>
       <c r="O74" s="4"/>
       <c r="P74" s="4"/>
@@ -7702,46 +7716,46 @@
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="1" t="s">
-        <v>744</v>
+        <v>749</v>
       </c>
       <c r="B75" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>750</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="G75" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="C75" s="2" t="s">
-        <v>745</v>
-      </c>
-      <c r="D75" s="2" t="s">
+      <c r="H75" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>751</v>
+      </c>
+      <c r="J75" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="E75" s="2" t="s">
+      <c r="K75" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="F75" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="G75" s="2" t="s">
+      <c r="L75" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="H75" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="I75" s="3" t="s">
-        <v>746</v>
-      </c>
-      <c r="J75" s="2" t="s">
+      <c r="M75" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="N75" s="5" t="s">
         <v>394</v>
-      </c>
-      <c r="K75" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="L75" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="M75" s="2" t="s">
-        <v>747</v>
-      </c>
-      <c r="N75" s="5" t="s">
-        <v>398</v>
       </c>
       <c r="O75" s="4"/>
       <c r="P75" s="4"/>
@@ -7759,20 +7773,48 @@
       <c r="AB75" s="4"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="32"/>
-      <c r="B76" s="4"/>
-      <c r="C76" s="4"/>
-      <c r="D76" s="4"/>
-      <c r="E76" s="4"/>
-      <c r="F76" s="4"/>
-      <c r="G76" s="4"/>
-      <c r="H76" s="4"/>
-      <c r="I76" s="4"/>
-      <c r="J76" s="4"/>
-      <c r="K76" s="4"/>
-      <c r="L76" s="4"/>
-      <c r="M76" s="4"/>
-      <c r="N76" s="4"/>
+      <c r="A76" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>753</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>754</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="K76" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="L76" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="M76" s="2" t="s">
+        <v>755</v>
+      </c>
+      <c r="N76" s="5" t="s">
+        <v>406</v>
+      </c>
       <c r="O76" s="4"/>
       <c r="P76" s="4"/>
       <c r="Q76" s="4"/>
@@ -7818,7 +7860,7 @@
       <c r="AA77" s="4"/>
       <c r="AB77" s="4"/>
     </row>
-    <row r="78" ht="15.75" hidden="1" customHeight="1">
+    <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="32"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -13759,34 +13801,34 @@
       <c r="AB275" s="4"/>
     </row>
     <row r="276" ht="15.75" hidden="1" customHeight="1">
-      <c r="A276" s="33"/>
-      <c r="B276" s="33"/>
-      <c r="C276" s="33"/>
-      <c r="D276" s="33"/>
-      <c r="E276" s="33"/>
-      <c r="F276" s="33"/>
-      <c r="G276" s="33"/>
-      <c r="H276" s="33"/>
-      <c r="I276" s="33"/>
-      <c r="J276" s="33"/>
-      <c r="K276" s="33"/>
-      <c r="L276" s="33"/>
-      <c r="M276" s="33"/>
-      <c r="N276" s="33"/>
-      <c r="O276" s="33"/>
-      <c r="P276" s="33"/>
-      <c r="Q276" s="33"/>
-      <c r="R276" s="33"/>
-      <c r="S276" s="33"/>
-      <c r="T276" s="33"/>
-      <c r="U276" s="33"/>
-      <c r="V276" s="33"/>
-      <c r="W276" s="33"/>
-      <c r="X276" s="33"/>
-      <c r="Y276" s="33"/>
-      <c r="Z276" s="33"/>
-      <c r="AA276" s="33"/>
-      <c r="AB276" s="33"/>
+      <c r="A276" s="32"/>
+      <c r="B276" s="4"/>
+      <c r="C276" s="4"/>
+      <c r="D276" s="4"/>
+      <c r="E276" s="4"/>
+      <c r="F276" s="4"/>
+      <c r="G276" s="4"/>
+      <c r="H276" s="4"/>
+      <c r="I276" s="4"/>
+      <c r="J276" s="4"/>
+      <c r="K276" s="4"/>
+      <c r="L276" s="4"/>
+      <c r="M276" s="4"/>
+      <c r="N276" s="4"/>
+      <c r="O276" s="4"/>
+      <c r="P276" s="4"/>
+      <c r="Q276" s="4"/>
+      <c r="R276" s="4"/>
+      <c r="S276" s="4"/>
+      <c r="T276" s="4"/>
+      <c r="U276" s="4"/>
+      <c r="V276" s="4"/>
+      <c r="W276" s="4"/>
+      <c r="X276" s="4"/>
+      <c r="Y276" s="4"/>
+      <c r="Z276" s="4"/>
+      <c r="AA276" s="4"/>
+      <c r="AB276" s="4"/>
     </row>
     <row r="277" ht="15.75" hidden="1" customHeight="1">
       <c r="A277" s="33"/>
@@ -35808,6 +35850,36 @@
       <c r="AA1010" s="33"/>
       <c r="AB1010" s="33"/>
     </row>
+    <row r="1011" ht="15.75" hidden="1" customHeight="1">
+      <c r="A1011" s="33"/>
+      <c r="B1011" s="33"/>
+      <c r="C1011" s="33"/>
+      <c r="D1011" s="33"/>
+      <c r="E1011" s="33"/>
+      <c r="F1011" s="33"/>
+      <c r="G1011" s="33"/>
+      <c r="H1011" s="33"/>
+      <c r="I1011" s="33"/>
+      <c r="J1011" s="33"/>
+      <c r="K1011" s="33"/>
+      <c r="L1011" s="33"/>
+      <c r="M1011" s="33"/>
+      <c r="N1011" s="33"/>
+      <c r="O1011" s="33"/>
+      <c r="P1011" s="33"/>
+      <c r="Q1011" s="33"/>
+      <c r="R1011" s="33"/>
+      <c r="S1011" s="33"/>
+      <c r="T1011" s="33"/>
+      <c r="U1011" s="33"/>
+      <c r="V1011" s="33"/>
+      <c r="W1011" s="33"/>
+      <c r="X1011" s="33"/>
+      <c r="Y1011" s="33"/>
+      <c r="Z1011" s="33"/>
+      <c r="AA1011" s="33"/>
+      <c r="AB1011" s="33"/>
+    </row>
   </sheetData>
   <printOptions gridLines="1" horizontalCentered="1"/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>